<commit_message>
Add shipper and VAT fields for KUEHNE_NAGEL supplier
Shipper reuses the already-reliable consignee value (same pattern as
DSV), since the SHIPPER field in the side-by-side CONSIGNEE/SHIPPER
block always matches INVOICE TO in observed samples. VAT is extracted
from the SUBTOTAL IDR line rather than the trailing digit on the item
charge line, which is actually a VAT-rate footnote reference code, not
an amount.

Also corrects 3 stale DD.MM.YYYY date cells in the two newly uploaded
reference fixtures to the current DD Mon YYYY format before installing
them as test samples.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JhL7qxuxZLsZyoRKZr1of6
</commit_message>
<xml_diff>
--- a/test_samples/KUEHNE_NAGEL/sample1_ref.xlsx
+++ b/test_samples/KUEHNE_NAGEL/sample1_ref.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="819" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="6510" yWindow="9375" windowWidth="28800" windowHeight="15315" tabRatio="819" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DWIHARTA" sheetId="1" state="visible" r:id="rId1"/>
@@ -507,24 +507,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
+  <dimension ref="A1:R12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
-    <col width="17.36328125" customWidth="1" style="8" min="1" max="1"/>
-    <col width="15.7265625" customWidth="1" style="8" min="2" max="2"/>
-    <col width="29.453125" customWidth="1" style="8" min="3" max="3"/>
+    <col width="17.375" customWidth="1" style="8" min="1" max="1"/>
+    <col width="15.75" customWidth="1" style="8" min="2" max="2"/>
+    <col width="29.5" customWidth="1" style="8" min="3" max="3"/>
     <col width="26" customWidth="1" style="8" min="4" max="4"/>
-    <col width="25.453125" bestFit="1" customWidth="1" style="8" min="5" max="5"/>
-    <col width="17.90625" customWidth="1" style="8" min="6" max="6"/>
-    <col width="29.26953125" customWidth="1" style="8" min="7" max="7"/>
-    <col width="13.7265625" customWidth="1" style="8" min="8" max="9"/>
-    <col width="17.6328125" customWidth="1" style="8" min="10" max="10"/>
-    <col width="20" customWidth="1" style="8" min="11" max="11"/>
-    <col width="16.90625" bestFit="1" customWidth="1" style="8" min="12" max="12"/>
-    <col width="18.6328125" bestFit="1" customWidth="1" style="8" min="13" max="13"/>
-    <col width="16.36328125" customWidth="1" style="8" min="14" max="14"/>
-    <col width="7.6328125" bestFit="1" customWidth="1" style="8" min="15" max="15"/>
-    <col width="15.08984375" bestFit="1" customWidth="1" style="8" min="16" max="16"/>
+    <col width="25.5" bestFit="1" customWidth="1" style="8" min="5" max="5"/>
+    <col width="17.875" customWidth="1" style="8" min="6" max="7"/>
+    <col width="29.25" customWidth="1" style="8" min="8" max="8"/>
+    <col width="13.75" customWidth="1" style="8" min="9" max="10"/>
+    <col width="17.625" customWidth="1" style="8" min="11" max="11"/>
+    <col width="20" customWidth="1" style="8" min="12" max="12"/>
+    <col width="16.875" bestFit="1" customWidth="1" style="8" min="13" max="13"/>
+    <col width="18.625" bestFit="1" customWidth="1" style="8" min="14" max="14"/>
+    <col width="16.375" customWidth="1" style="8" min="15" max="15"/>
+    <col width="7.625" bestFit="1" customWidth="1" style="8" min="16" max="16"/>
+    <col width="15.125" bestFit="1" customWidth="1" style="8" min="17" max="17"/>
+    <col width="13.375" customWidth="1" style="8" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="45" customFormat="1" customHeight="1" s="1">
@@ -566,63 +567,74 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
+          <t>VAT</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
           <t>Order No.</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Arrive Date
 到達日</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>on board date
 開船日</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>B/L NO.
 提單號碼</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>MBL NO.
 主提單號碼</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Port of Loading
 啟運港</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>Port of discharge
 目的港</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>Volume
 材積</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>Vessel
 船名</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>Container no.
 貨櫃號碼</t>
         </is>
       </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>Shipper
+出貨方</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
@@ -653,88 +665,96 @@
       <c r="F2" s="4" t="n">
         <v>1521098</v>
       </c>
-      <c r="G2" s="0" t="inlineStr">
+      <c r="G2" s="4" t="n">
+        <v>167321</v>
+      </c>
+      <c r="H2" s="0" t="inlineStr">
         <is>
           <t>RYH0810074280</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>12 Oct 2026</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>23 Aug 2026</t>
         </is>
       </c>
-      <c r="J2" s="0" t="n">
+      <c r="K2" s="0" t="n">
         <v>1076510528</v>
       </c>
-      <c r="K2" s="0" t="inlineStr">
+      <c r="L2" s="0" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="L2" s="0" t="inlineStr">
+      <c r="M2" s="0" t="inlineStr">
         <is>
           <t>JAKARTA</t>
         </is>
       </c>
-      <c r="M2" s="7" t="inlineStr">
+      <c r="N2" s="7" t="inlineStr">
         <is>
           <t>Los Angeles</t>
         </is>
       </c>
-      <c r="N2" s="0" t="n">
+      <c r="O2" s="0" t="n">
         <v>11.81</v>
       </c>
-      <c r="O2" s="0" t="inlineStr">
+      <c r="P2" s="0" t="inlineStr">
         <is>
           <t>CMA CGM WHITE SHARK</t>
         </is>
       </c>
-      <c r="P2" s="0" t="inlineStr">
+      <c r="Q2" s="0" t="inlineStr">
         <is>
           <t>N/A</t>
+        </is>
+      </c>
+      <c r="R2" s="0" t="inlineStr">
+        <is>
+          <t>PT. POU YUEN INDONESIA</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
       <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
       <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
       <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
-      <c r="H7" s="3" t="n"/>
       <c r="I7" s="3" t="n"/>
+      <c r="J7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="n"/>
+      <c r="J8" s="3" t="n"/>
     </row>
     <row r="9"/>
     <row r="10"/>
     <row r="11"/>
     <row r="12">
-      <c r="Q12" s="1" t="n"/>
+      <c r="R12" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
KUEHNE NAGEL: supplier from footer, FCL containers/volume, PO NO fallback
- SUPPLIER taken from the KN invoice bottom-right footer (Faktur Pajak is
  not always attached); Faktur seller name kept as fallback
- Container no. from the line above each "SEAL NO."; FCL Volume is the
  aggregated container count (e.g. 1X40G+1X40H+1X20G), LCL keeps VOL
- Order No. falls back to the "PO NO." list when there is no
  COMMERCIAL INVOICE NUMBER
- VAT row Description is "VAT"
- Currency no longer hard-coded to IDR; amounts may carry decimals;
  grand total also accepts "AMOUNT DUE"
- Update KN reference answers (sample3 from the user's new Excel)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_samples/KUEHNE_NAGEL/sample1_ref.xlsx
+++ b/test_samples/KUEHNE_NAGEL/sample1_ref.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="6855" yWindow="2535" windowWidth="28800" windowHeight="15510" tabRatio="819" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DWIHARTA" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="DWIHARTA" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -726,6 +726,11 @@
           <t>PT. POU YUEN INDONESIA</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>VAT</t>
+        </is>
+      </c>
       <c r="G3" s="4" t="n">
         <v>167321</v>
       </c>

</xml_diff>